<commit_message>
🎯 Strike: drop mostbetfrance.com from p6 (Corsearch says account exists), remove bisect files
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brand-protection/2026-09-28/strike/01-mono_other-p6.xlsx
+++ b/brand-protection/2026-09-28/strike/01-mono_other-p6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M201"/>
+  <dimension ref="A1:M200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1153,7 +1153,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://mostbetfrance.com/</t>
+          <t>https://mostbetgiris-az.it.com/</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1173,14 +1173,14 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mostbetfrance.com</t>
+          <t>mostbetgiris-az.it.com</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://mostbetgiris-az.it.com/</t>
+          <t>https://mostbetgirisitesi.com/</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1200,14 +1200,14 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>mostbetgiris-az.it.com</t>
+          <t>mostbetgirisitesi.com</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://mostbetgirisitesi.com/</t>
+          <t>https://mostbeticefishing.com/</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1227,14 +1227,14 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>mostbetgirisitesi.com</t>
+          <t>mostbeticefishing.com</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://mostbeticefishing.com/</t>
+          <t>https://mostbetjoga-pt.com/</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1254,14 +1254,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mostbeticefishing.com</t>
+          <t>mostbetjoga-pt.com</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://mostbetjoga-pt.com/</t>
+          <t>https://mostbetkaszino-hungary.com/</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1281,14 +1281,14 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>mostbetjoga-pt.com</t>
+          <t>mostbetkaszino-hungary.com</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://mostbetkaszino-hungary.com/</t>
+          <t>https://mostbetkaszino.net/</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1301,21 +1301,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>mostbetkaszino-hungary.com</t>
+          <t>mostbetkaszino.net</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://mostbetkaszino.net/</t>
+          <t>https://mostbetkazino-top.ru/</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1328,16 +1323,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>mostbetkaszino.net</t>
+          <t>mostbetkazino-top.ru</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://mostbetkazino-top.ru/</t>
+          <t>https://mostbetkazinotop.ru/</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1357,14 +1357,14 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>mostbetkazino-top.ru</t>
+          <t>mostbetkazinotop.ru</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://mostbetkazinotop.ru/</t>
+          <t>https://mostbetluckyjetpredictor.com/</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1379,19 +1379,19 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>mostbetkazinotop.ru</t>
+          <t>mostbetluckyjetpredictor.com</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://mostbetluckyjetpredictor.com/</t>
+          <t>https://mostbetminespredictor.com/</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>mostbetluckyjetpredictor.com</t>
+          <t>mostbetminespredictor.com</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://mostbetminespredictor.com/</t>
+          <t>https://mostbetn.com/</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1438,14 +1438,14 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mostbetminespredictor.com</t>
+          <t>mostbetn.com</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://mostbetn.com/</t>
+          <t>https://mostbetnederland.nl/</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1460,19 +1460,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>mostbetn.com</t>
+          <t>mostbetnederland.nl</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://mostbetnederland.nl/</t>
+          <t>https://mostbetnl.com/</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1487,19 +1487,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>mostbetnederland.nl</t>
+          <t>mostbetnl.com</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://mostbetnl.com/</t>
+          <t>https://mostbetofficial.nl/</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1514,19 +1514,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>mostbetnl.com</t>
+          <t>mostbetofficial.nl</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://mostbetofficial.nl/</t>
+          <t>https://mostbetonline-kz.com/</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1541,19 +1541,19 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>mostbetofficial.nl</t>
+          <t>mostbetonline-kz.com</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://mostbetonline-kz.com/</t>
+          <t>https://mostbetonline.art/</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1566,21 +1566,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>mostbetonline-kz.com</t>
+          <t>mostbetonline.art</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://mostbetonline.art/</t>
+          <t>https://mostbetonline.ro/</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1593,16 +1588,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>mostbetonline.art</t>
+          <t>mostbetonline.ro</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://mostbetonline.ro/</t>
+          <t>https://mostbetplaytr.com/</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1617,19 +1617,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>mostbetonline.ro</t>
+          <t>mostbetplaytr.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://mostbetplaytr.com/</t>
+          <t>https://mostbetplaywin7-95.ru/</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1644,19 +1644,19 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>mostbetplaytr.com</t>
+          <t>mostbetplaywin7-95.ru</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://mostbetplaywin7-95.ru/</t>
+          <t>https://mostbetplinko.com/</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1671,19 +1671,19 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>mostbetplaywin7-95.ru</t>
+          <t>mostbetplinko.com</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://mostbetplinko.com/</t>
+          <t>https://mostbetpolska.com.pl/</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1698,19 +1698,19 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>mostbetplinko.com</t>
+          <t>mostbetpolska.com.pl</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://mostbetpolska.com.pl/</t>
+          <t>https://mostbetpolskacasino.com/</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1725,19 +1725,19 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>mostbetpolska.com.pl</t>
+          <t>mostbetpolskacasino.com</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://mostbetpolskacasino.com/</t>
+          <t>https://mostbetportugal.site/</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1750,21 +1750,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>mostbetpolskacasino.com</t>
+          <t>mostbetportugal.site</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://mostbetportugal.site/</t>
+          <t>https://mostbetportuguese.com/</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1777,16 +1772,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>mostbetportugal.site</t>
+          <t>mostbetportuguese.com</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://mostbetportuguese.com/</t>
+          <t>https://mostbetqo.com/</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1806,14 +1806,14 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>mostbetportuguese.com</t>
+          <t>mostbetqo.com</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://mostbetqo.com/</t>
+          <t>https://mostbetrtp.com/</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1833,14 +1833,14 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>mostbetqo.com</t>
+          <t>mostbetrtp.com</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://mostbetrtp.com/</t>
+          <t>https://mostbets-bk1.ru/</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1855,19 +1855,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>mostbetrtp.com</t>
+          <t>mostbets-bk1.ru</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://mostbets-bk1.ru/</t>
+          <t>https://mostbets-casino.ro/</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1882,19 +1882,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>mostbets-bk1.ru</t>
+          <t>mostbets-casino.ro</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://mostbets-casino.ro/</t>
+          <t>https://mostbets-cz.net/</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1907,21 +1907,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>mostbets-casino.ro</t>
+          <t>mostbets-cz.net</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://mostbets-cz.net/</t>
+          <t>https://mostbets-czech.org/</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1936,14 +1931,14 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>mostbets-cz.net</t>
+          <t>mostbets-czech.org</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://mostbets-czech.org/</t>
+          <t>https://mostbets-deutschland.de/</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1956,16 +1951,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>mostbets-czech.org</t>
+          <t>mostbets-deutschland.de</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://mostbets-deutschland.de/</t>
+          <t>https://mostbets-hu.org/</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1978,21 +1978,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>mostbets-deutschland.de</t>
+          <t>mostbets-hu.org</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://mostbets-hu.org/</t>
+          <t>https://mostbets-magyar.com/</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2005,16 +2000,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>mostbets-hu.org</t>
+          <t>mostbets-magyar.com</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://mostbets-magyar.com/</t>
+          <t>https://mostbets-magyar.net/</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2027,21 +2027,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>mostbets-magyar.com</t>
+          <t>mostbets-magyar.net</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://mostbets-magyar.net/</t>
+          <t>https://mostbets-online.cz/</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2054,16 +2049,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>mostbets-magyar.net</t>
+          <t>mostbets-online.cz</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://mostbets-online.cz/</t>
+          <t>https://mostbets-online.org/</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2076,21 +2076,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>mostbets-online.cz</t>
+          <t>mostbets-online.org</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://mostbets-online.org/</t>
+          <t>https://mostbets-pl-casino-com.pl/</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2103,16 +2098,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>mostbets-online.org</t>
+          <t>mostbets-pl-casino-com.pl</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://mostbets-pl-casino-com.pl/</t>
+          <t>https://mostbets-poland.com.pl/</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2132,14 +2132,14 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>mostbets-pl-casino-com.pl</t>
+          <t>mostbets-poland.com.pl</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://mostbets-poland.com.pl/</t>
+          <t>https://mostbets-polska.com.pl/</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2159,14 +2159,14 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>mostbets-poland.com.pl</t>
+          <t>mostbets-polska.com.pl</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://mostbets-polska.com.pl/</t>
+          <t>https://mostbets-portugal.com/</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2181,19 +2181,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>mostbets-polska.com.pl</t>
+          <t>mostbets-portugal.com</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://mostbets-portugal.com/</t>
+          <t>https://mostbets.agro.pl/</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2208,19 +2208,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>mostbets-portugal.com</t>
+          <t>mostbets.agro.pl</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://mostbets.agro.pl/</t>
+          <t>https://mostbets.auto.pl/</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2240,14 +2240,14 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>mostbets.agro.pl</t>
+          <t>mostbets.auto.pl</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://mostbets.auto.pl/</t>
+          <t>https://mostbets.fr/</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2262,19 +2262,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>mostbets.auto.pl</t>
+          <t>mostbets.fr</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://mostbets.fr/</t>
+          <t>https://mostbets.games/</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2287,21 +2287,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>mostbets.fr</t>
+          <t>mostbets.games</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://mostbets.games/</t>
+          <t>https://mostbets.poker/</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2316,14 +2311,14 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>mostbets.games</t>
+          <t>mostbets.poker</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://mostbets.poker/</t>
+          <t>https://mostbets.ro/</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2336,16 +2331,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>mostbets.poker</t>
+          <t>mostbets.ro</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://mostbets.ro/</t>
+          <t>https://mostbets.tech/</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2358,21 +2358,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>mostbets.ro</t>
+          <t>mostbets.tech</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://mostbets.tech/</t>
+          <t>https://mostbets1.com/</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2385,16 +2380,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>mostbets.tech</t>
+          <t>mostbets1.com</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://mostbets1.com/</t>
+          <t>https://mostbetscasino.ro/</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>mostbets1.com</t>
+          <t>mostbetscasino.ro</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://mostbetscasino.ro/</t>
+          <t>https://mostbetsite.app/</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2434,21 +2434,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>mostbetscasino.ro</t>
+          <t>mostbetsite.app</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://mostbetsite.app/</t>
+          <t>https://mostbetslots.com.de/</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2461,16 +2456,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>mostbetsite.app</t>
+          <t>mostbetslots.com.de</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://mostbetslots.com.de/</t>
+          <t>https://mostbetslotsnet.click/</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2483,21 +2483,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>mostbetslots.com.de</t>
+          <t>mostbetslotsnet.click</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://mostbetslotsnet.click/</t>
+          <t>https://mostbetslovenske.com/</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2510,16 +2505,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>mostbetslotsnet.click</t>
+          <t>mostbetslovenske.com</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://mostbetslovenske.com/</t>
+          <t>https://mostbetsportfogadas.com/</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>mostbetslovenske.com</t>
+          <t>mostbetsportfogadas.com</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://mostbetsportfogadas.com/</t>
+          <t>https://mostbett-cz.cz/</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2561,19 +2561,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>mostbetsportfogadas.com</t>
+          <t>mostbett-cz.cz</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://mostbett-cz.cz/</t>
+          <t>https://mostbett.de/</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2588,19 +2588,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>mostbett-cz.cz</t>
+          <t>mostbett.de</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://mostbett.de/</t>
+          <t>https://mostbett.ro/</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2615,19 +2615,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>mostbett.de</t>
+          <t>mostbett.ro</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://mostbett.ro/</t>
+          <t>https://mostbetting.casino/</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2640,21 +2640,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>mostbett.ro</t>
+          <t>mostbetting.casino</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://mostbetting.casino/</t>
+          <t>https://mostbetting.games/</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2669,14 +2664,14 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>mostbetting.casino</t>
+          <t>mostbetting.games</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://mostbetting.games/</t>
+          <t>https://mostbetting.ltd/</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2691,14 +2686,14 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>mostbetting.games</t>
+          <t>mostbetting.ltd</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://mostbetting.ltd/</t>
+          <t>https://mostbettop.net/</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2713,14 +2708,14 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>mostbetting.ltd</t>
+          <t>mostbettop.net</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://mostbettop.net/</t>
+          <t>https://mostbettor.com/</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2733,16 +2728,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>mostbettop.net</t>
+          <t>mostbettor.com</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://mostbettor.com/</t>
+          <t>https://mostbettor.games/</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2755,21 +2755,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>mostbettor.com</t>
+          <t>mostbettor.games</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://mostbettor.games/</t>
+          <t>https://mostbettowerrush.com/</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2782,16 +2777,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>mostbettor.games</t>
+          <t>mostbettowerrush.com</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://mostbettowerrush.com/</t>
+          <t>https://mostbettr-slots.store/</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2804,21 +2804,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>mostbettowerrush.com</t>
+          <t>mostbettr-slots.store</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://mostbettr-slots.store/</t>
+          <t>https://mostbetuzbets.com/</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2831,16 +2826,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>mostbettr-slots.store</t>
+          <t>mostbetuzbets.com</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://mostbetuzbets.com/</t>
+          <t>https://mostbetviptr.com/</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2860,14 +2860,14 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>mostbetuzbets.com</t>
+          <t>mostbetviptr.com</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://mostbetviptr.com/</t>
+          <t>https://mostbetviva-it.com/</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2887,14 +2887,14 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>mostbetviptr.com</t>
+          <t>mostbetviva-it.com</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://mostbetviva-it.com/</t>
+          <t>https://mostbetwin-cz.com/</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2914,14 +2914,14 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>mostbetviva-it.com</t>
+          <t>mostbetwin-cz.com</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://mostbetwin-cz.com/</t>
+          <t>https://mostbetwin-mx.com/</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2941,14 +2941,14 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>mostbetwin-cz.com</t>
+          <t>mostbetwin-mx.com</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://mostbetwin-mx.com/</t>
+          <t>https://mostbetwinpl.com/</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2968,14 +2968,14 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>mostbetwin-mx.com</t>
+          <t>mostbetwinpl.com</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://mostbetwinpl.com/</t>
+          <t>https://mostbetwinturkey.com/</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2995,14 +2995,14 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>mostbetwinpl.com</t>
+          <t>mostbetwinturkey.com</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://mostbetwinturkey.com/</t>
+          <t>https://mostbetwithdrawal.com/</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3022,14 +3022,14 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>mostbetwinturkey.com</t>
+          <t>mostbetwithdrawal.com</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://mostbetwithdrawal.com/</t>
+          <t>https://mostbetz.pt/</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3044,19 +3044,19 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>mostbetwithdrawal.com</t>
+          <t>mostbetz.pt</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://mostbetz.pt/</t>
+          <t>https://mostbetzerkalorab.ru/</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3071,19 +3071,19 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>mostbetz.pt</t>
+          <t>mostbetzerkalorab.ru</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://mostbetzerkalorab.ru/</t>
+          <t>https://mostfunpillows.com/</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3098,19 +3098,19 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>mostbetzerkalorab.ru</t>
+          <t>mostfunpillows.com</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://mostfunpillows.com/</t>
+          <t>https://mostplays.net/</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3123,21 +3123,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>mostfunpillows.com</t>
+          <t>mostplays.net</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://mostplays.net/</t>
+          <t>https://mstbt-amp-forab.ru/</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3150,16 +3145,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>mostplays.net</t>
+          <t>mstbt-amp-forab.ru</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://mstbt-amp-forab.ru/</t>
+          <t>https://mstbt-amp-sibir.ru/</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3179,14 +3179,14 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>mstbt-amp-forab.ru</t>
+          <t>mstbt-amp-sibir.ru</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://mstbt-amp-sibir.ru/</t>
+          <t>https://mstbt-amp-vesta.ru/</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3206,14 +3206,14 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>mstbt-amp-sibir.ru</t>
+          <t>mstbt-amp-vesta.ru</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://mstbt-amp-vesta.ru/</t>
+          <t>https://murphsgaslight.com/</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3228,19 +3228,19 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>mstbt-amp-vesta.ru</t>
+          <t>murphsgaslight.com</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://murphsgaslight.com/</t>
+          <t>https://museodeburgos.com/</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3260,14 +3260,14 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>murphsgaslight.com</t>
+          <t>museodeburgos.com</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://museodeburgos.com/</t>
+          <t>https://museumantiquities.tj/</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3282,19 +3282,19 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>museodeburgos.com</t>
+          <t>museumantiquities.tj</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://museumantiquities.tj/</t>
+          <t>https://mycomfypad.com/</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3309,19 +3309,19 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>museumantiquities.tj</t>
+          <t>mycomfypad.com</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://mycomfypad.com/</t>
+          <t>https://mypdapp.com/</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3341,14 +3341,14 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>mycomfypad.com</t>
+          <t>mypdapp.com</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://mypdapp.com/</t>
+          <t>https://myrmecos.net/</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3361,21 +3361,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>mypdapp.com</t>
+          <t>myrmecos.net</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>https://myrmecos.net/</t>
+          <t>https://nadpartner.ru/</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3388,16 +3383,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>myrmecos.net</t>
+          <t>nadpartner.ru</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>https://nadpartner.ru/</t>
+          <t>https://nailsprof.ru/</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3417,14 +3417,14 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>nadpartner.ru</t>
+          <t>nailsprof.ru</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>https://nailsprof.ru/</t>
+          <t>https://napelemes-futes.hu/</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3439,19 +3439,19 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>HU</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>nailsprof.ru</t>
+          <t>napelemes-futes.hu</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>https://napelemes-futes.hu/</t>
+          <t>https://napitkitop.ru/</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3466,19 +3466,19 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>HU</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>napelemes-futes.hu</t>
+          <t>napitkitop.ru</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>https://napitkitop.ru/</t>
+          <t>https://nationalparty.com.pk/</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3493,19 +3493,19 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>napitkitop.ru</t>
+          <t>nationalparty.com.pk</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>https://nationalparty.com.pk/</t>
+          <t>https://nature-prod.ru/</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3520,19 +3520,19 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>nationalparty.com.pk</t>
+          <t>nature-prod.ru</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>https://nature-prod.ru/</t>
+          <t>https://netdaycompass.org/</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3545,21 +3545,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>nature-prod.ru</t>
+          <t>netdaycompass.org</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://netdaycompass.org/</t>
+          <t>https://netflorista.com/</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3572,16 +3567,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>netdaycompass.org</t>
+          <t>netflorista.com</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>https://netflorista.com/</t>
+          <t>https://netpoulsafe.eu/</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3594,21 +3594,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>netflorista.com</t>
+          <t>netpoulsafe.eu</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>https://netpoulsafe.eu/</t>
+          <t>https://newlepnina.ru/</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3621,16 +3616,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>netpoulsafe.eu</t>
+          <t>newlepnina.ru</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>https://newlepnina.ru/</t>
+          <t>https://news-mostbet-tr.com/</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3645,19 +3645,19 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>newlepnina.ru</t>
+          <t>news-mostbet-tr.com</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://news-mostbet-tr.com/</t>
+          <t>https://newsart.net/</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3670,21 +3670,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>news-mostbet-tr.com</t>
+          <t>newsart.net</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>https://newsart.net/</t>
+          <t>https://newsforb2b.com/</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3697,16 +3692,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>newsart.net</t>
+          <t>newsforb2b.com</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>https://newsforb2b.com/</t>
+          <t>https://nicolasroy.pro/</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3719,21 +3719,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>newsforb2b.com</t>
+          <t>nicolasroy.pro</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>https://nicolasroy.pro/</t>
+          <t>https://nigerianports.org/</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3748,14 +3743,14 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>nicolasroy.pro</t>
+          <t>nigerianports.org</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://nigerianports.org/</t>
+          <t>https://nika-kosmetika.ru/</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3768,16 +3763,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>nigerianports.org</t>
+          <t>nika-kosmetika.ru</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://nika-kosmetika.ru/</t>
+          <t>https://njzhenguyan.ru/</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3797,14 +3797,14 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>nika-kosmetika.ru</t>
+          <t>njzhenguyan.ru</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://njzhenguyan.ru/</t>
+          <t>https://nl-mostbet.com/</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3819,19 +3819,19 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>njzhenguyan.ru</t>
+          <t>nl-mostbet.com</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://nl-mostbet.com/</t>
+          <t>https://nodosele.cfd/</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3844,21 +3844,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>nl-mostbet.com</t>
+          <t>nodosele.cfd</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://nodosele.cfd/</t>
+          <t>https://nodosele.com/</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3871,16 +3866,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>nodosele.cfd</t>
+          <t>nodosele.com</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>https://nodosele.com/</t>
+          <t>https://non-stopdogwear.cz/</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3895,19 +3895,19 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>nodosele.com</t>
+          <t>non-stopdogwear.cz</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>https://non-stopdogwear.cz/</t>
+          <t>https://nord-kross.ru/</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3922,19 +3922,19 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>non-stopdogwear.cz</t>
+          <t>nord-kross.ru</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>https://nord-kross.ru/</t>
+          <t>https://noticiasdocavado.pt/</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3949,19 +3949,19 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>nord-kross.ru</t>
+          <t>noticiasdocavado.pt</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>https://noticiasdocavado.pt/</t>
+          <t>https://novadon.ru/</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3976,19 +3976,19 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>noticiasdocavado.pt</t>
+          <t>novadon.ru</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>https://novadon.ru/</t>
+          <t>https://nr-sibiria.ru/</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -4008,14 +4008,14 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>novadon.ru</t>
+          <t>nr-sibiria.ru</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>https://nr-sibiria.ru/</t>
+          <t>https://nz-yalta.ru/</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -4035,14 +4035,14 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>nr-sibiria.ru</t>
+          <t>nz-yalta.ru</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>https://nz-yalta.ru/</t>
+          <t>https://oakmapper.org/</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -4055,21 +4055,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>nz-yalta.ru</t>
+          <t>oakmapper.org</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>https://oakmapper.org/</t>
+          <t>https://oboi5.ru/</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -4082,16 +4077,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>oakmapper.org</t>
+          <t>oboi5.ru</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>https://oboi5.ru/</t>
+          <t>https://obserwatorzy.org/</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -4104,21 +4104,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>oboi5.ru</t>
+          <t>obserwatorzy.org</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>https://obserwatorzy.org/</t>
+          <t>https://ofbirdandcagegame.com/</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -4131,16 +4126,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>obserwatorzy.org</t>
+          <t>ofbirdandcagegame.com</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>https://ofbirdandcagegame.com/</t>
+          <t>https://official-mostbet.online/</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -4153,21 +4153,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>ofbirdandcagegame.com</t>
+          <t>official-mostbet.online</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>https://official-mostbet.online/</t>
+          <t>https://ohlook.in/</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -4180,16 +4175,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>official-mostbet.online</t>
+          <t>ohlook.in</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://ohlook.in/</t>
+          <t>https://ojura.org/</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -4202,21 +4202,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>ohlook.in</t>
+          <t>ojura.org</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://ojura.org/</t>
+          <t>https://olln.org/</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4231,14 +4226,14 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>ojura.org</t>
+          <t>olln.org</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>https://olln.org/</t>
+          <t>https://one-pravo.ru/</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4251,16 +4246,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>olln.org</t>
+          <t>one-pravo.ru</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>https://one-pravo.ru/</t>
+          <t>https://online-amp-best129.cfd/</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4273,21 +4273,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>one-pravo.ru</t>
+          <t>online-amp-best129.cfd</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>https://online-amp-best129.cfd/</t>
+          <t>https://online-amp-best263.cfd/</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4302,14 +4297,14 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>online-amp-best129.cfd</t>
+          <t>online-amp-best263.cfd</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>https://online-amp-best263.cfd/</t>
+          <t>https://online-game-best529.cfd/</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4324,14 +4319,14 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>online-amp-best263.cfd</t>
+          <t>online-game-best529.cfd</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>https://online-game-best529.cfd/</t>
+          <t>https://online-game-top826.cfd/</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4346,14 +4341,14 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>online-game-best529.cfd</t>
+          <t>online-game-top826.cfd</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>https://online-game-top826.cfd/</t>
+          <t>https://online-super-amp503.cfd/</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4368,14 +4363,14 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>online-game-top826.cfd</t>
+          <t>online-super-amp503.cfd</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>https://online-super-amp503.cfd/</t>
+          <t>https://online-super-game926.cfd/</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4390,14 +4385,14 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>online-super-amp503.cfd</t>
+          <t>online-super-game926.cfd</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>https://online-super-game926.cfd/</t>
+          <t>https://online-super-top482.cfd/</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4412,14 +4407,14 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>online-super-game926.cfd</t>
+          <t>online-super-top482.cfd</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>https://online-super-top482.cfd/</t>
+          <t>https://online-top-best-29.cfd/</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4434,14 +4429,14 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>online-super-top482.cfd</t>
+          <t>online-top-best-29.cfd</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>https://online-top-best-29.cfd/</t>
+          <t>https://online-top-super860.cfd/</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4456,14 +4451,14 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>online-top-best-29.cfd</t>
+          <t>online-top-super860.cfd</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>https://online-top-super860.cfd/</t>
+          <t>https://onlinemostbet.ink/</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4478,14 +4473,14 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>online-top-super860.cfd</t>
+          <t>onlinemostbet.ink</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>https://onlinemostbet.ink/</t>
+          <t>https://onlinemostbet.online/</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4500,14 +4495,14 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>onlinemostbet.ink</t>
+          <t>onlinemostbet.online</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>https://onlinemostbet.online/</t>
+          <t>https://opk-gorodu.ru/</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4520,16 +4515,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>onlinemostbet.online</t>
+          <t>opk-gorodu.ru</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>https://opk-gorodu.ru/</t>
+          <t>https://optimistic-theatre.ru/</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4549,14 +4549,14 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>opk-gorodu.ru</t>
+          <t>optimistic-theatre.ru</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>https://optimistic-theatre.ru/</t>
+          <t>https://orangecosmetics.ru/</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4576,14 +4576,14 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>optimistic-theatre.ru</t>
+          <t>orangecosmetics.ru</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>https://orangecosmetics.ru/</t>
+          <t>https://orient-watches.ru/</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4603,14 +4603,14 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>orangecosmetics.ru</t>
+          <t>orient-watches.ru</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>https://orient-watches.ru/</t>
+          <t>https://otilor-shop.ru/</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4630,14 +4630,14 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>orient-watches.ru</t>
+          <t>otilor-shop.ru</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>https://otilor-shop.ru/</t>
+          <t>https://ousterhout.net/</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4650,21 +4650,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>otilor-shop.ru</t>
+          <t>ousterhout.net</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>https://ousterhout.net/</t>
+          <t>https://outdoormoviehq.com/</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4677,16 +4672,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>ousterhout.net</t>
+          <t>outdoormoviehq.com</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>https://outdoormoviehq.com/</t>
+          <t>https://owpd.eu/</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4699,21 +4699,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>outdoormoviehq.com</t>
+          <t>owpd.eu</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>https://owpd.eu/</t>
+          <t>https://ozogpytlak.pl/</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4726,16 +4721,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>owpd.eu</t>
+          <t>ozogpytlak.pl</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>https://ozogpytlak.pl/</t>
+          <t>https://packardevents.org/</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4748,21 +4748,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>ozogpytlak.pl</t>
+          <t>packardevents.org</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>https://packardevents.org/</t>
+          <t>https://panamera63detailing.ru/</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4775,16 +4770,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>packardevents.org</t>
+          <t>panamera63detailing.ru</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>https://panamera63detailing.ru/</t>
+          <t>https://partnerupak.ru/</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4804,14 +4804,14 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>panamera63detailing.ru</t>
+          <t>partnerupak.ru</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>https://partnerupak.ru/</t>
+          <t>https://parts-portal.ru/</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4831,14 +4831,14 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>partnerupak.ru</t>
+          <t>parts-portal.ru</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>https://parts-portal.ru/</t>
+          <t>https://partymania-krd.ru/</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4858,14 +4858,14 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>parts-portal.ru</t>
+          <t>partymania-krd.ru</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>https://partymania-krd.ru/</t>
+          <t>https://paterfamilia.ru/</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4885,14 +4885,14 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>partymania-krd.ru</t>
+          <t>paterfamilia.ru</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>https://paterfamilia.ru/</t>
+          <t>https://patriar.ru/</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4912,14 +4912,14 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>paterfamilia.ru</t>
+          <t>patriar.ru</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>https://patriar.ru/</t>
+          <t>https://paywatches.net/</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4932,21 +4932,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>patriar.ru</t>
+          <t>paywatches.net</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>https://paywatches.net/</t>
+          <t>https://paywatchesnet.cfd/</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4961,14 +4956,14 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>paywatches.net</t>
+          <t>paywatchesnet.cfd</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>https://paywatchesnet.cfd/</t>
+          <t>https://peixe-eletrico.com/</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4981,16 +4976,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>paywatchesnet.cfd</t>
+          <t>peixe-eletrico.com</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>https://peixe-eletrico.com/</t>
+          <t>https://peppymom.ru/</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -5005,19 +5005,19 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>peixe-eletrico.com</t>
+          <t>peppymom.ru</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>https://peppymom.ru/</t>
+          <t>https://perpendox.com/</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -5032,19 +5032,19 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>peppymom.ru</t>
+          <t>perpendox.com</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>https://perpendox.com/</t>
+          <t>https://peswithyou.com/</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -5064,14 +5064,14 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>perpendox.com</t>
+          <t>peswithyou.com</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>https://peswithyou.com/</t>
+          <t>https://petesuen.com/</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -5091,14 +5091,14 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>peswithyou.com</t>
+          <t>petesuen.com</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>https://petesuen.com/</t>
+          <t>https://pggrupp.ru/</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -5113,19 +5113,19 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>petesuen.com</t>
+          <t>pggrupp.ru</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>https://pggrupp.ru/</t>
+          <t>https://photorism.ru/</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -5145,14 +5145,14 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>pggrupp.ru</t>
+          <t>photorism.ru</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>https://photorism.ru/</t>
+          <t>https://pingvi-pizza.ru/</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -5172,14 +5172,14 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>photorism.ru</t>
+          <t>pingvi-pizza.ru</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>https://pingvi-pizza.ru/</t>
+          <t>https://pisa.com.pk/</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -5194,19 +5194,19 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>pingvi-pizza.ru</t>
+          <t>pisa.com.pk</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>https://pisa.com.pk/</t>
+          <t>https://pl-20-kotlas.ru/</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5221,19 +5221,19 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>pisa.com.pk</t>
+          <t>pl-20-kotlas.ru</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>https://pl-20-kotlas.ru/</t>
+          <t>https://pl-mostbet-casino.pl/</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5248,19 +5248,19 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>pl-20-kotlas.ru</t>
+          <t>pl-mostbet-casino.pl</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>https://pl-mostbet-casino.pl/</t>
+          <t>https://pl-mostbet.pl/</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5280,14 +5280,14 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>pl-mostbet-casino.pl</t>
+          <t>pl-mostbet.pl</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>https://pl-mostbet.pl/</t>
+          <t>https://play-game-best194.cfd/</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5300,21 +5300,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>pl-mostbet.pl</t>
+          <t>play-game-best194.cfd</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>https://play-game-best194.cfd/</t>
+          <t>https://play-top-best237.cfd/</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5329,14 +5324,14 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>play-game-best194.cfd</t>
+          <t>play-top-best237.cfd</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>https://play-top-best237.cfd/</t>
+          <t>https://play-top-super572.cfd/</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5351,14 +5346,14 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>play-top-best237.cfd</t>
+          <t>play-top-super572.cfd</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>https://play-top-super572.cfd/</t>
+          <t>https://playmostbetbd.com/</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5371,16 +5366,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p6</t>
         </is>
       </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>play-top-super572.cfd</t>
+          <t>playmostbetbd.com</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>https://playmostbetbd.com/</t>
+          <t>https://plm-engineering.ru/</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5395,19 +5395,19 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>playmostbetbd.com</t>
+          <t>plm-engineering.ru</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>https://plm-engineering.ru/</t>
+          <t>https://ploshka-ceramic.ru/</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5427,14 +5427,14 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>plm-engineering.ru</t>
+          <t>ploshka-ceramic.ru</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>https://ploshka-ceramic.ru/</t>
+          <t>https://plumberinbelmont247.com/</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5449,19 +5449,19 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>ploshka-ceramic.ru</t>
+          <t>plumberinbelmont247.com</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>https://plumberinbelmont247.com/</t>
+          <t>https://plumberinhalfmoonbay247.com/</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5481,14 +5481,14 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>plumberinbelmont247.com</t>
+          <t>plumberinhalfmoonbay247.com</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>https://plumberinhalfmoonbay247.com/</t>
+          <t>https://plumberinrosemont247.com/</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5508,14 +5508,14 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>plumberinhalfmoonbay247.com</t>
+          <t>plumberinrosemont247.com</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>https://plumberinrosemont247.com/</t>
+          <t>https://plumberinsananselmo247.com/</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5535,14 +5535,14 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>plumberinrosemont247.com</t>
+          <t>plumberinsananselmo247.com</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>https://plumberinsananselmo247.com/</t>
+          <t>https://plumbermountainview247.com/</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5561,33 +5561,6 @@
         </is>
       </c>
       <c r="E200" t="inlineStr">
-        <is>
-          <t>plumberinsananselmo247.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>https://plumbermountainview247.com/</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>Trademark Infringement</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>strike-01-mono-other,strike-01-mono-other-p6</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
-      <c r="E201" t="inlineStr">
         <is>
           <t>plumbermountainview247.com</t>
         </is>

</xml_diff>